<commit_message>
add VKCT 2026 results, update configuration and calendar
</commit_message>
<xml_diff>
--- a/processor/outputTemplate.xlsx
+++ b/processor/outputTemplate.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Template" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Template!$B$2:$R$200</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Template!$B$2:$R$175</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Template!$B$2:$Z$200</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Template!$B$2:$Z$175</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area_0_0" vbProcedure="false">Template!$B$2:$N$71</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area_0_0_0" vbProcedure="false">Template!$B$2:$N$50</definedName>
   </definedNames>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="33">
   <si>
     <t xml:space="preserve">Force Valašskokarpatská cyklotour</t>
   </si>
@@ -46,19 +46,31 @@
     <t xml:space="preserve">Bratřejovské kotáry</t>
   </si>
   <si>
+    <t xml:space="preserve">O pohár starosty obce Lačnov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XC Cup Napajedla</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ploština - Memoriál Josefa Valčíka</t>
   </si>
   <si>
-    <t xml:space="preserve">24. 5.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14. 6.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9. 8.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. 10.</t>
+    <t xml:space="preserve">23. 5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13. 6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. 8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">???</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. 9.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. 10.</t>
   </si>
   <si>
     <t xml:space="preserve">Jméno</t>
@@ -79,10 +91,22 @@
     <t xml:space="preserve">pořadí po 2. závodě</t>
   </si>
   <si>
+    <t xml:space="preserve">3. závod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pořadí po 3. závodě</t>
+  </si>
+  <si>
     <t xml:space="preserve">4. závod</t>
   </si>
   <si>
     <t xml:space="preserve">pořadí po 4. závodě</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. závod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pořadí po 5. závodě</t>
   </si>
   <si>
     <t xml:space="preserve">6. závod</t>
@@ -110,7 +134,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -147,6 +171,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="1"/>
     </font>
     <font>
@@ -253,7 +284,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -278,6 +309,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -290,31 +325,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -449,15 +484,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A2:R8"/>
+  <dimension ref="A2:Z8"/>
   <sheetFormatPr defaultColWidth="8.8671875" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1012" min="1009" style="1" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16376" min="16373" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16380" min="16377" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1020" min="1017" style="1" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -473,7 +506,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="R2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
@@ -513,156 +546,232 @@
       <c r="P4" s="5"/>
       <c r="Q4" s="5"/>
       <c r="R4" s="5"/>
+      <c r="S4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="X4" s="5"/>
+      <c r="Y4" s="5"/>
+      <c r="Z4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7" t="s">
+      <c r="F5" s="8"/>
+      <c r="G5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7"/>
-      <c r="R5" s="7"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="T5" s="8"/>
+      <c r="U5" s="8"/>
+      <c r="V5" s="8"/>
+      <c r="W5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="X5" s="8"/>
+      <c r="Y5" s="8"/>
+      <c r="Z5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8"/>
-      <c r="B6" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="11" t="s">
+      <c r="A6" s="9"/>
+      <c r="B6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="11"/>
-      <c r="I6" s="10" t="s">
+      <c r="C6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="10"/>
-      <c r="K6" s="11" t="s">
+      <c r="D6" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="N6" s="10"/>
-      <c r="O6" s="11" t="s">
+      <c r="F6" s="11"/>
+      <c r="G6" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="10" t="s">
+      <c r="H6" s="12"/>
+      <c r="I6" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="R6" s="10"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="L6" s="12"/>
+      <c r="M6" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="N6" s="11"/>
+      <c r="O6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="R6" s="11"/>
+      <c r="S6" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="T6" s="12"/>
+      <c r="U6" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="V6" s="11"/>
+      <c r="W6" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="X6" s="12"/>
+      <c r="Y6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="K7" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="L7" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="M7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="N7" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="O7" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="P7" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q7" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="R7" s="12" t="s">
-        <v>22</v>
+      <c r="A7" s="9"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="N7" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="O7" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="P7" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q7" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="R7" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="S7" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="T7" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="U7" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="V7" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="W7" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y7" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z7" s="13" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="17"/>
-      <c r="Q8" s="12"/>
-      <c r="R8" s="16"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="13"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="17"/>
+      <c r="O8" s="14"/>
+      <c r="P8" s="18"/>
+      <c r="Q8" s="13"/>
+      <c r="R8" s="17"/>
+      <c r="S8" s="14"/>
+      <c r="T8" s="18"/>
+      <c r="U8" s="13"/>
+      <c r="V8" s="17"/>
+      <c r="W8" s="14"/>
+      <c r="X8" s="18"/>
+      <c r="Y8" s="13"/>
+      <c r="Z8" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="28">
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B3:J3"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="K4:N4"/>
     <mergeCell ref="O4:R4"/>
+    <mergeCell ref="S4:V4"/>
+    <mergeCell ref="W4:Z4"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:J5"/>
     <mergeCell ref="K5:N5"/>
     <mergeCell ref="O5:R5"/>
+    <mergeCell ref="S5:V5"/>
+    <mergeCell ref="W5:Z5"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="D6:D7"/>
@@ -673,13 +782,18 @@
     <mergeCell ref="M6:N6"/>
     <mergeCell ref="O6:P6"/>
     <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="U6:V6"/>
+    <mergeCell ref="W6:X6"/>
+    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="R2" r:id="rId1" display="https://vkct.webnode.cz/"/>
+    <hyperlink ref="Z2" r:id="rId1" display="https://vkct.webnode.cz/"/>
     <hyperlink ref="E4" r:id="rId2" display="Hradní okruh"/>
     <hyperlink ref="G4" r:id="rId3" display="Klobucká kola"/>
     <hyperlink ref="K4" r:id="rId4" display="Bratřejovské kotáry"/>
-    <hyperlink ref="O4" r:id="rId5" display="Ploština - Memoriál Josefa Valčíka"/>
+    <hyperlink ref="O4" r:id="rId5" display="O pohár starosty obce Lačnov"/>
+    <hyperlink ref="W4" r:id="rId6" display="Ploština - Memoriál Josefa Valčíka"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.329861111111111" right="0.329861111111111" top="0.329861111111111" bottom="0.329861111111111" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>